<commit_message>
S2 restructure: question-node + Excel Table as main path, flow as advanced
- Main finding: question-node(File) + Excel Table alone enables orchestrator analysis on all channels; no flow needed for the common case.

- s02-excel-analysis: 2-track overview with honest cost/benefit.

- Rename s02-1-excel-flow.md -> s02-1-excel-question.md: topic + question-node(File) + A/B compare 과일판매.xlsx (Table) vs 과일판매_raw.xlsx (raw).

- Rename s02-2-excel-topic.md -> s02-2-excel-flow-advanced.md: flow + Office Script + AI Prompt with explicit when-it-helps/when-it-hurts + code-interpreter ON/OFF + data-schema requirement.

- Assets: add 과일판매_raw.xlsx; apply Excel Table 'FruitSales' (A1:D193) to 과일판매.xlsx.

- Cross-refs updated: advanced-course.md, s03-3-integrate.md, s06-1-excel-knowledge.md.
</commit_message>
<xml_diff>
--- a/assets/files/과일판매.xlsx
+++ b/assets/files/과일판매.xlsx
@@ -146,6 +146,19 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FruitSales" displayName="FruitSales" ref="A1:D193" headerRowCount="1">
+  <autoFilter ref="A1:D193"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="연도"/>
+    <tableColumn id="2" name="분기"/>
+    <tableColumn id="3" name="과일"/>
+    <tableColumn id="4" name="판매량"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3926,11 +3939,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Privileged" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>